<commit_message>
fix timetable download styling
</commit_message>
<xml_diff>
--- a/backend/export_templates/campion_timetable_export_template.xlsx
+++ b/backend/export_templates/campion_timetable_export_template.xlsx
@@ -18,7 +18,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="h:mm Am/Pm"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -159,10 +159,23 @@
     <font>
       <name val="Trebuchet MS"/>
       <b val="1"/>
+      <color rgb="FF660033"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Trebuchet MS"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Trebuchet MS"/>
+      <b val="1"/>
+      <color rgb="FFcc9900"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -229,13 +242,8 @@
         <fgColor rgb="FFbfbfbf"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="107">
+  <borders count="102">
     <border>
       <left/>
       <right/>
@@ -1516,131 +1524,107 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFc6c6c6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFc6c6c6"/>
+      </bottom>
+    </border>
+    <border>
       <left style="medium">
         <color rgb="FF000000"/>
       </left>
       <right style="thin">
-        <color rgb="FFC6C6C6"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFc6c6c6"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC6C6C6"/>
+      <left style="thin">
+        <color rgb="FFc6c6c6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC6C6C6"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC6C6C6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC6C6C6"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFC6C6C6"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFC6C6C6"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFC6C6C6"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFC6C6C6"/>
+        <color rgb="FFc6c6c6"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="20" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="97" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="198">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2156,19 +2140,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="69" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="97" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="100" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="104" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="98" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="97" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="99" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="99" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="103" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="106" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="101" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -2192,8 +2176,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="71" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="86" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="12">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="tt_class_HIS" xfId="1" hidden="0"/>
+    <cellStyle name="tt_class_THE" xfId="2" hidden="0"/>
+    <cellStyle name="tt_class_LIT" xfId="3" hidden="0"/>
+    <cellStyle name="tt_class_PHI" xfId="4" hidden="0"/>
+    <cellStyle name="tt_class_GRE" xfId="5" hidden="0"/>
+    <cellStyle name="tt_class_LAN" xfId="6" hidden="0"/>
+    <cellStyle name="tt_class_default" xfId="7" hidden="0"/>
+    <cellStyle name="tt_block_gold" xfId="8" hidden="0"/>
+    <cellStyle name="tt_block_blue" xfId="9" hidden="0"/>
+    <cellStyle name="tt_block_pink" xfId="10" hidden="0"/>
+    <cellStyle name="tt_block_unnamed" xfId="11" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>

</xml_diff>

<commit_message>
fix: enhance Excel export template fidelity and uniformity
- Refactor `build_template.py` to ensure every room×slot band in the timetable Excel export has a uniform empty look, with specific fills for each day type (white for Tuesday/Thursday, grey for Monday/Wednesday/Friday) and a consistent medium box border on all sides.
- Update the `_blank_grid` function to reset all grid bands uniformly, improving visual consistency and eliminating gaps.
- Modify the `_class_named_style` and `_block_named_style` functions to apply the new uniform border style across all named styles.
- Revise tests in `test_96_excel_export_style_parity.py` to validate the new uniformity in grid box styles and ensure that all cells adhere to the expected styling derived from the template.
- Update documentation to reflect changes in the Excel export process and styling rules, ensuring clarity on the new uniformity and fidelity to the original template.
</commit_message>
<xml_diff>
--- a/backend/export_templates/campion_timetable_export_template.xlsx
+++ b/backend/export_templates/campion_timetable_export_template.xlsx
@@ -403,7 +403,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="78">
+  <borders count="79">
     <border>
       <left/>
       <right/>
@@ -1372,44 +1372,58 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="8" borderId="70" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="8" borderId="78" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="22" borderId="70" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="6" borderId="70" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="22" borderId="78" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="6" borderId="78" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="71" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="78" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="491">
+  <cellXfs count="442">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -2973,153 +2987,32 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="30" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="71" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="72" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="71" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="4" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="2" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="72" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="78" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="78" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="31" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="71" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="30" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="70" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="72" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="78" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="78" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="32" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="34" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="71" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="35" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="70" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
@@ -3136,50 +3029,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="67" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="71" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="71" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="30" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="36" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="3" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="35" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="70" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="8" borderId="33" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0" hidden="0"/>
@@ -3188,6 +3037,15 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -3994,45 +3852,45 @@
         </is>
       </c>
       <c r="B6" s="423" t="n"/>
-      <c r="C6" s="424" t="n"/>
-      <c r="D6" s="424" t="n"/>
-      <c r="E6" s="425" t="n"/>
-      <c r="F6" s="425" t="n"/>
-      <c r="G6" s="425" t="n"/>
-      <c r="H6" s="425" t="n"/>
-      <c r="I6" s="426" t="n"/>
-      <c r="J6" s="427" t="n"/>
-      <c r="K6" s="428" t="n"/>
-      <c r="L6" s="156" t="n"/>
-      <c r="M6" s="428" t="n"/>
-      <c r="N6" s="429" t="n"/>
-      <c r="O6" s="430" t="n"/>
-      <c r="P6" s="428" t="n"/>
-      <c r="Q6" s="431" t="n"/>
-      <c r="R6" s="432" t="n"/>
-      <c r="S6" s="425" t="n"/>
-      <c r="T6" s="424" t="n"/>
-      <c r="U6" s="433" t="n"/>
-      <c r="V6" s="433" t="n"/>
-      <c r="W6" s="425" t="n"/>
-      <c r="X6" s="425" t="n"/>
-      <c r="Y6" s="434" t="n"/>
-      <c r="Z6" s="427" t="n"/>
-      <c r="AA6" s="428" t="n"/>
-      <c r="AB6" s="429" t="n"/>
-      <c r="AC6" s="429" t="n"/>
-      <c r="AD6" s="430" t="n"/>
-      <c r="AE6" s="428" t="n"/>
-      <c r="AF6" s="428" t="n"/>
-      <c r="AG6" s="431" t="n"/>
-      <c r="AH6" s="435" t="n"/>
-      <c r="AI6" s="425" t="n"/>
-      <c r="AJ6" s="436" t="n"/>
-      <c r="AK6" s="152" t="n"/>
-      <c r="AL6" s="151" t="n"/>
-      <c r="AM6" s="424" t="n"/>
-      <c r="AN6" s="425" t="n"/>
-      <c r="AO6" s="426" t="n"/>
+      <c r="C6" s="423" t="n"/>
+      <c r="D6" s="423" t="n"/>
+      <c r="E6" s="423" t="n"/>
+      <c r="F6" s="423" t="n"/>
+      <c r="G6" s="423" t="n"/>
+      <c r="H6" s="423" t="n"/>
+      <c r="I6" s="423" t="n"/>
+      <c r="J6" s="424" t="n"/>
+      <c r="K6" s="424" t="n"/>
+      <c r="L6" s="424" t="n"/>
+      <c r="M6" s="424" t="n"/>
+      <c r="N6" s="424" t="n"/>
+      <c r="O6" s="424" t="n"/>
+      <c r="P6" s="424" t="n"/>
+      <c r="Q6" s="424" t="n"/>
+      <c r="R6" s="423" t="n"/>
+      <c r="S6" s="423" t="n"/>
+      <c r="T6" s="423" t="n"/>
+      <c r="U6" s="423" t="n"/>
+      <c r="V6" s="423" t="n"/>
+      <c r="W6" s="423" t="n"/>
+      <c r="X6" s="423" t="n"/>
+      <c r="Y6" s="423" t="n"/>
+      <c r="Z6" s="424" t="n"/>
+      <c r="AA6" s="424" t="n"/>
+      <c r="AB6" s="424" t="n"/>
+      <c r="AC6" s="424" t="n"/>
+      <c r="AD6" s="424" t="n"/>
+      <c r="AE6" s="424" t="n"/>
+      <c r="AF6" s="424" t="n"/>
+      <c r="AG6" s="424" t="n"/>
+      <c r="AH6" s="423" t="n"/>
+      <c r="AI6" s="423" t="n"/>
+      <c r="AJ6" s="423" t="n"/>
+      <c r="AK6" s="423" t="n"/>
+      <c r="AL6" s="423" t="n"/>
+      <c r="AM6" s="423" t="n"/>
+      <c r="AN6" s="423" t="n"/>
+      <c r="AO6" s="423" t="n"/>
       <c r="AP6" s="422" t="inlineStr">
         <is>
           <t>9.00 AM - 9.50 AM</t>
@@ -4040,192 +3898,192 @@
       </c>
     </row>
     <row r="7" ht="45.6" customHeight="1" thickBot="1">
-      <c r="A7" s="437" t="n"/>
-      <c r="B7" s="438" t="n"/>
-      <c r="C7" s="439" t="n"/>
-      <c r="D7" s="439" t="n"/>
-      <c r="E7" s="440" t="n"/>
-      <c r="F7" s="440" t="n"/>
-      <c r="G7" s="440" t="n"/>
-      <c r="H7" s="440" t="n"/>
-      <c r="I7" s="441" t="n"/>
-      <c r="J7" s="442" t="n"/>
-      <c r="K7" s="440" t="n"/>
-      <c r="L7" s="443" t="n"/>
-      <c r="M7" s="440" t="n"/>
-      <c r="N7" s="444" t="n"/>
-      <c r="O7" s="439" t="n"/>
-      <c r="P7" s="440" t="n"/>
-      <c r="Q7" s="441" t="n"/>
-      <c r="R7" s="441" t="n"/>
-      <c r="S7" s="440" t="n"/>
-      <c r="T7" s="439" t="n"/>
-      <c r="U7" s="440" t="n"/>
-      <c r="V7" s="440" t="n"/>
-      <c r="W7" s="440" t="n"/>
-      <c r="X7" s="440" t="n"/>
-      <c r="Y7" s="441" t="n"/>
-      <c r="Z7" s="442" t="n"/>
-      <c r="AA7" s="440" t="n"/>
-      <c r="AB7" s="444" t="n"/>
-      <c r="AC7" s="444" t="n"/>
-      <c r="AD7" s="439" t="n"/>
-      <c r="AE7" s="440" t="n"/>
-      <c r="AF7" s="440" t="n"/>
-      <c r="AG7" s="441" t="n"/>
-      <c r="AH7" s="442" t="n"/>
-      <c r="AI7" s="440" t="n"/>
-      <c r="AJ7" s="444" t="n"/>
-      <c r="AK7" s="443" t="n"/>
+      <c r="A7" s="425" t="n"/>
+      <c r="B7" s="421" t="n"/>
+      <c r="C7" s="421" t="n"/>
+      <c r="D7" s="421" t="n"/>
+      <c r="E7" s="421" t="n"/>
+      <c r="F7" s="421" t="n"/>
+      <c r="G7" s="421" t="n"/>
+      <c r="H7" s="421" t="n"/>
+      <c r="I7" s="421" t="n"/>
+      <c r="J7" s="421" t="n"/>
+      <c r="K7" s="421" t="n"/>
+      <c r="L7" s="421" t="n"/>
+      <c r="M7" s="421" t="n"/>
+      <c r="N7" s="421" t="n"/>
+      <c r="O7" s="421" t="n"/>
+      <c r="P7" s="421" t="n"/>
+      <c r="Q7" s="421" t="n"/>
+      <c r="R7" s="421" t="n"/>
+      <c r="S7" s="421" t="n"/>
+      <c r="T7" s="421" t="n"/>
+      <c r="U7" s="421" t="n"/>
+      <c r="V7" s="421" t="n"/>
+      <c r="W7" s="421" t="n"/>
+      <c r="X7" s="421" t="n"/>
+      <c r="Y7" s="421" t="n"/>
+      <c r="Z7" s="421" t="n"/>
+      <c r="AA7" s="421" t="n"/>
+      <c r="AB7" s="421" t="n"/>
+      <c r="AC7" s="421" t="n"/>
+      <c r="AD7" s="421" t="n"/>
+      <c r="AE7" s="421" t="n"/>
+      <c r="AF7" s="421" t="n"/>
+      <c r="AG7" s="421" t="n"/>
+      <c r="AH7" s="421" t="n"/>
+      <c r="AI7" s="421" t="n"/>
+      <c r="AJ7" s="421" t="n"/>
+      <c r="AK7" s="421" t="n"/>
       <c r="AL7" s="421" t="n"/>
-      <c r="AM7" s="439" t="n"/>
-      <c r="AN7" s="440" t="n"/>
-      <c r="AO7" s="441" t="n"/>
-      <c r="AP7" s="437" t="n"/>
+      <c r="AM7" s="421" t="n"/>
+      <c r="AN7" s="421" t="n"/>
+      <c r="AO7" s="421" t="n"/>
+      <c r="AP7" s="425" t="n"/>
     </row>
     <row r="8" ht="45.6" customHeight="1">
-      <c r="A8" s="445" t="inlineStr">
+      <c r="A8" s="426" t="inlineStr">
         <is>
           <t>10.00 AM - 10.50 AM</t>
         </is>
       </c>
-      <c r="B8" s="446" t="n"/>
-      <c r="C8" s="447" t="n"/>
-      <c r="D8" s="424" t="n"/>
-      <c r="E8" s="425" t="n"/>
-      <c r="F8" s="425" t="n"/>
-      <c r="G8" s="425" t="n"/>
-      <c r="H8" s="425" t="n"/>
-      <c r="I8" s="426" t="n"/>
-      <c r="J8" s="448" t="n"/>
-      <c r="K8" s="449" t="n"/>
-      <c r="L8" s="156" t="n"/>
-      <c r="M8" s="450" t="n"/>
-      <c r="N8" s="429" t="n"/>
-      <c r="O8" s="430" t="n"/>
-      <c r="P8" s="430" t="n"/>
-      <c r="Q8" s="431" t="n"/>
-      <c r="R8" s="432" t="n"/>
-      <c r="S8" s="451" t="n"/>
-      <c r="T8" s="424" t="n"/>
-      <c r="U8" s="436" t="n"/>
-      <c r="V8" s="433" t="n"/>
-      <c r="W8" s="424" t="n"/>
-      <c r="X8" s="425" t="n"/>
-      <c r="Y8" s="154" t="n"/>
-      <c r="Z8" s="427" t="n"/>
-      <c r="AA8" s="428" t="n"/>
-      <c r="AB8" s="430" t="n"/>
-      <c r="AC8" s="452" t="n"/>
-      <c r="AD8" s="428" t="n"/>
-      <c r="AE8" s="428" t="n"/>
-      <c r="AF8" s="428" t="n"/>
-      <c r="AG8" s="431" t="n"/>
-      <c r="AH8" s="435" t="n"/>
-      <c r="AI8" s="425" t="n"/>
-      <c r="AJ8" s="436" t="n"/>
-      <c r="AK8" s="453" t="n"/>
-      <c r="AL8" s="454" t="n"/>
-      <c r="AM8" s="424" t="n"/>
-      <c r="AN8" s="425" t="n"/>
-      <c r="AO8" s="426" t="n"/>
-      <c r="AP8" s="445" t="inlineStr">
+      <c r="B8" s="427" t="n"/>
+      <c r="C8" s="427" t="n"/>
+      <c r="D8" s="423" t="n"/>
+      <c r="E8" s="423" t="n"/>
+      <c r="F8" s="423" t="n"/>
+      <c r="G8" s="423" t="n"/>
+      <c r="H8" s="423" t="n"/>
+      <c r="I8" s="423" t="n"/>
+      <c r="J8" s="424" t="n"/>
+      <c r="K8" s="424" t="n"/>
+      <c r="L8" s="424" t="n"/>
+      <c r="M8" s="428" t="n"/>
+      <c r="N8" s="424" t="n"/>
+      <c r="O8" s="424" t="n"/>
+      <c r="P8" s="424" t="n"/>
+      <c r="Q8" s="424" t="n"/>
+      <c r="R8" s="423" t="n"/>
+      <c r="S8" s="427" t="n"/>
+      <c r="T8" s="423" t="n"/>
+      <c r="U8" s="423" t="n"/>
+      <c r="V8" s="423" t="n"/>
+      <c r="W8" s="423" t="n"/>
+      <c r="X8" s="423" t="n"/>
+      <c r="Y8" s="423" t="n"/>
+      <c r="Z8" s="424" t="n"/>
+      <c r="AA8" s="424" t="n"/>
+      <c r="AB8" s="424" t="n"/>
+      <c r="AC8" s="428" t="n"/>
+      <c r="AD8" s="424" t="n"/>
+      <c r="AE8" s="424" t="n"/>
+      <c r="AF8" s="424" t="n"/>
+      <c r="AG8" s="424" t="n"/>
+      <c r="AH8" s="423" t="n"/>
+      <c r="AI8" s="423" t="n"/>
+      <c r="AJ8" s="423" t="n"/>
+      <c r="AK8" s="427" t="n"/>
+      <c r="AL8" s="427" t="n"/>
+      <c r="AM8" s="423" t="n"/>
+      <c r="AN8" s="423" t="n"/>
+      <c r="AO8" s="423" t="n"/>
+      <c r="AP8" s="426" t="inlineStr">
         <is>
           <t>10.00 AM - 10.50 AM</t>
         </is>
       </c>
     </row>
     <row r="9" ht="45.95" customHeight="1" thickBot="1">
-      <c r="A9" s="437" t="n"/>
-      <c r="B9" s="455" t="n"/>
-      <c r="C9" s="456" t="n"/>
-      <c r="D9" s="439" t="n"/>
-      <c r="E9" s="440" t="n"/>
-      <c r="F9" s="440" t="n"/>
-      <c r="G9" s="440" t="n"/>
-      <c r="H9" s="440" t="n"/>
-      <c r="I9" s="441" t="n"/>
-      <c r="J9" s="438" t="n"/>
+      <c r="A9" s="425" t="n"/>
+      <c r="B9" s="429" t="n"/>
+      <c r="C9" s="429" t="n"/>
+      <c r="D9" s="421" t="n"/>
+      <c r="E9" s="421" t="n"/>
+      <c r="F9" s="421" t="n"/>
+      <c r="G9" s="421" t="n"/>
+      <c r="H9" s="421" t="n"/>
+      <c r="I9" s="421" t="n"/>
+      <c r="J9" s="421" t="n"/>
       <c r="K9" s="421" t="n"/>
-      <c r="L9" s="443" t="n"/>
-      <c r="M9" s="457" t="n"/>
-      <c r="N9" s="444" t="n"/>
-      <c r="O9" s="439" t="n"/>
-      <c r="P9" s="439" t="n"/>
-      <c r="Q9" s="441" t="n"/>
-      <c r="R9" s="441" t="n"/>
-      <c r="S9" s="457" t="n"/>
-      <c r="T9" s="439" t="n"/>
-      <c r="U9" s="444" t="n"/>
-      <c r="V9" s="440" t="n"/>
-      <c r="W9" s="439" t="n"/>
-      <c r="X9" s="440" t="n"/>
-      <c r="Y9" s="458" t="n"/>
-      <c r="Z9" s="442" t="n"/>
-      <c r="AA9" s="440" t="n"/>
-      <c r="AB9" s="439" t="n"/>
-      <c r="AC9" s="459" t="n"/>
-      <c r="AD9" s="440" t="n"/>
-      <c r="AE9" s="440" t="n"/>
-      <c r="AF9" s="440" t="n"/>
-      <c r="AG9" s="441" t="n"/>
-      <c r="AH9" s="442" t="n"/>
-      <c r="AI9" s="440" t="n"/>
-      <c r="AJ9" s="444" t="n"/>
-      <c r="AK9" s="460" t="n"/>
-      <c r="AL9" s="461" t="n"/>
-      <c r="AM9" s="439" t="n"/>
-      <c r="AN9" s="440" t="n"/>
-      <c r="AO9" s="441" t="n"/>
-      <c r="AP9" s="437" t="n"/>
+      <c r="L9" s="421" t="n"/>
+      <c r="M9" s="429" t="n"/>
+      <c r="N9" s="421" t="n"/>
+      <c r="O9" s="421" t="n"/>
+      <c r="P9" s="421" t="n"/>
+      <c r="Q9" s="421" t="n"/>
+      <c r="R9" s="421" t="n"/>
+      <c r="S9" s="429" t="n"/>
+      <c r="T9" s="421" t="n"/>
+      <c r="U9" s="421" t="n"/>
+      <c r="V9" s="421" t="n"/>
+      <c r="W9" s="421" t="n"/>
+      <c r="X9" s="421" t="n"/>
+      <c r="Y9" s="421" t="n"/>
+      <c r="Z9" s="421" t="n"/>
+      <c r="AA9" s="421" t="n"/>
+      <c r="AB9" s="421" t="n"/>
+      <c r="AC9" s="429" t="n"/>
+      <c r="AD9" s="421" t="n"/>
+      <c r="AE9" s="421" t="n"/>
+      <c r="AF9" s="421" t="n"/>
+      <c r="AG9" s="421" t="n"/>
+      <c r="AH9" s="421" t="n"/>
+      <c r="AI9" s="421" t="n"/>
+      <c r="AJ9" s="421" t="n"/>
+      <c r="AK9" s="429" t="n"/>
+      <c r="AL9" s="429" t="n"/>
+      <c r="AM9" s="421" t="n"/>
+      <c r="AN9" s="421" t="n"/>
+      <c r="AO9" s="421" t="n"/>
+      <c r="AP9" s="425" t="n"/>
     </row>
     <row r="10" ht="45.95" customHeight="1">
-      <c r="A10" s="462" t="inlineStr">
+      <c r="A10" s="430" t="inlineStr">
         <is>
           <t>11.00 AM - 11.50AM</t>
         </is>
       </c>
       <c r="B10" s="423" t="n"/>
-      <c r="C10" s="424" t="n"/>
-      <c r="D10" s="424" t="n"/>
-      <c r="E10" s="425" t="n"/>
-      <c r="F10" s="425" t="n"/>
-      <c r="G10" s="425" t="n"/>
-      <c r="H10" s="425" t="n"/>
-      <c r="I10" s="426" t="n"/>
-      <c r="J10" s="427" t="n"/>
-      <c r="K10" s="450" t="n"/>
-      <c r="L10" s="463" t="n"/>
-      <c r="M10" s="450" t="n"/>
-      <c r="N10" s="452" t="n"/>
-      <c r="O10" s="464" t="n"/>
-      <c r="P10" s="450" t="n"/>
-      <c r="Q10" s="465" t="n"/>
-      <c r="R10" s="432" t="n"/>
-      <c r="S10" s="451" t="n"/>
-      <c r="T10" s="466" t="n"/>
-      <c r="U10" s="433" t="n"/>
-      <c r="V10" s="433" t="n"/>
-      <c r="W10" s="424" t="n"/>
-      <c r="X10" s="425" t="n"/>
-      <c r="Y10" s="432" t="n"/>
-      <c r="Z10" s="467" t="n"/>
-      <c r="AA10" s="450" t="n"/>
-      <c r="AB10" s="430" t="n"/>
-      <c r="AC10" s="452" t="n"/>
-      <c r="AD10" s="428" t="n"/>
-      <c r="AE10" s="428" t="n"/>
-      <c r="AF10" s="428" t="n"/>
-      <c r="AG10" s="431" t="n"/>
-      <c r="AH10" s="435" t="n"/>
-      <c r="AI10" s="425" t="n"/>
-      <c r="AJ10" s="436" t="n"/>
-      <c r="AK10" s="453" t="n"/>
-      <c r="AL10" s="454" t="n"/>
-      <c r="AM10" s="424" t="n"/>
-      <c r="AN10" s="425" t="n"/>
-      <c r="AO10" s="426" t="n"/>
-      <c r="AP10" s="462" t="inlineStr">
+      <c r="C10" s="423" t="n"/>
+      <c r="D10" s="423" t="n"/>
+      <c r="E10" s="423" t="n"/>
+      <c r="F10" s="423" t="n"/>
+      <c r="G10" s="423" t="n"/>
+      <c r="H10" s="423" t="n"/>
+      <c r="I10" s="423" t="n"/>
+      <c r="J10" s="424" t="n"/>
+      <c r="K10" s="428" t="n"/>
+      <c r="L10" s="428" t="n"/>
+      <c r="M10" s="428" t="n"/>
+      <c r="N10" s="428" t="n"/>
+      <c r="O10" s="428" t="n"/>
+      <c r="P10" s="428" t="n"/>
+      <c r="Q10" s="428" t="n"/>
+      <c r="R10" s="423" t="n"/>
+      <c r="S10" s="427" t="n"/>
+      <c r="T10" s="423" t="n"/>
+      <c r="U10" s="423" t="n"/>
+      <c r="V10" s="423" t="n"/>
+      <c r="W10" s="423" t="n"/>
+      <c r="X10" s="423" t="n"/>
+      <c r="Y10" s="423" t="n"/>
+      <c r="Z10" s="428" t="n"/>
+      <c r="AA10" s="428" t="n"/>
+      <c r="AB10" s="424" t="n"/>
+      <c r="AC10" s="428" t="n"/>
+      <c r="AD10" s="424" t="n"/>
+      <c r="AE10" s="424" t="n"/>
+      <c r="AF10" s="424" t="n"/>
+      <c r="AG10" s="424" t="n"/>
+      <c r="AH10" s="423" t="n"/>
+      <c r="AI10" s="423" t="n"/>
+      <c r="AJ10" s="423" t="n"/>
+      <c r="AK10" s="427" t="n"/>
+      <c r="AL10" s="427" t="n"/>
+      <c r="AM10" s="423" t="n"/>
+      <c r="AN10" s="423" t="n"/>
+      <c r="AO10" s="423" t="n"/>
+      <c r="AP10" s="430" t="inlineStr">
         <is>
           <t>11.00 AM - 11.50AM</t>
         </is>
@@ -4233,50 +4091,50 @@
     </row>
     <row r="11" ht="45.95" customHeight="1" thickBot="1">
       <c r="A11" s="421" t="n"/>
-      <c r="B11" s="438" t="n"/>
-      <c r="C11" s="439" t="n"/>
-      <c r="D11" s="439" t="n"/>
-      <c r="E11" s="440" t="n"/>
-      <c r="F11" s="440" t="n"/>
-      <c r="G11" s="440" t="n"/>
-      <c r="H11" s="440" t="n"/>
-      <c r="I11" s="441" t="n"/>
-      <c r="J11" s="442" t="n"/>
-      <c r="K11" s="457" t="n"/>
-      <c r="L11" s="460" t="n"/>
-      <c r="M11" s="457" t="n"/>
-      <c r="N11" s="459" t="n"/>
-      <c r="O11" s="456" t="n"/>
-      <c r="P11" s="457" t="n"/>
-      <c r="Q11" s="468" t="n"/>
-      <c r="R11" s="441" t="n"/>
-      <c r="S11" s="457" t="n"/>
-      <c r="T11" s="469" t="n"/>
-      <c r="U11" s="440" t="n"/>
-      <c r="V11" s="440" t="n"/>
-      <c r="W11" s="439" t="n"/>
-      <c r="X11" s="440" t="n"/>
-      <c r="Y11" s="441" t="n"/>
-      <c r="Z11" s="470" t="n"/>
-      <c r="AA11" s="457" t="n"/>
-      <c r="AB11" s="439" t="n"/>
-      <c r="AC11" s="459" t="n"/>
-      <c r="AD11" s="440" t="n"/>
-      <c r="AE11" s="440" t="n"/>
-      <c r="AF11" s="440" t="n"/>
-      <c r="AG11" s="441" t="n"/>
-      <c r="AH11" s="442" t="n"/>
-      <c r="AI11" s="440" t="n"/>
-      <c r="AJ11" s="444" t="n"/>
-      <c r="AK11" s="460" t="n"/>
-      <c r="AL11" s="461" t="n"/>
-      <c r="AM11" s="439" t="n"/>
-      <c r="AN11" s="440" t="n"/>
-      <c r="AO11" s="441" t="n"/>
+      <c r="B11" s="421" t="n"/>
+      <c r="C11" s="421" t="n"/>
+      <c r="D11" s="421" t="n"/>
+      <c r="E11" s="421" t="n"/>
+      <c r="F11" s="421" t="n"/>
+      <c r="G11" s="421" t="n"/>
+      <c r="H11" s="421" t="n"/>
+      <c r="I11" s="421" t="n"/>
+      <c r="J11" s="421" t="n"/>
+      <c r="K11" s="429" t="n"/>
+      <c r="L11" s="429" t="n"/>
+      <c r="M11" s="429" t="n"/>
+      <c r="N11" s="429" t="n"/>
+      <c r="O11" s="429" t="n"/>
+      <c r="P11" s="429" t="n"/>
+      <c r="Q11" s="429" t="n"/>
+      <c r="R11" s="421" t="n"/>
+      <c r="S11" s="429" t="n"/>
+      <c r="T11" s="421" t="n"/>
+      <c r="U11" s="421" t="n"/>
+      <c r="V11" s="421" t="n"/>
+      <c r="W11" s="421" t="n"/>
+      <c r="X11" s="421" t="n"/>
+      <c r="Y11" s="421" t="n"/>
+      <c r="Z11" s="429" t="n"/>
+      <c r="AA11" s="429" t="n"/>
+      <c r="AB11" s="421" t="n"/>
+      <c r="AC11" s="429" t="n"/>
+      <c r="AD11" s="421" t="n"/>
+      <c r="AE11" s="421" t="n"/>
+      <c r="AF11" s="421" t="n"/>
+      <c r="AG11" s="421" t="n"/>
+      <c r="AH11" s="421" t="n"/>
+      <c r="AI11" s="421" t="n"/>
+      <c r="AJ11" s="421" t="n"/>
+      <c r="AK11" s="429" t="n"/>
+      <c r="AL11" s="429" t="n"/>
+      <c r="AM11" s="421" t="n"/>
+      <c r="AN11" s="421" t="n"/>
+      <c r="AO11" s="421" t="n"/>
       <c r="AP11" s="421" t="n"/>
     </row>
     <row r="12" ht="23.45" customHeight="1" thickBot="1">
-      <c r="A12" s="471" t="inlineStr">
+      <c r="A12" s="431" t="inlineStr">
         <is>
           <t>12.00 PM - 1.30PM</t>
         </is>
@@ -4286,62 +4144,62 @@
           <t>Mass/Lunch</t>
         </is>
       </c>
-      <c r="C12" s="472" t="n"/>
-      <c r="D12" s="472" t="n"/>
-      <c r="E12" s="472" t="n"/>
-      <c r="F12" s="472" t="n"/>
-      <c r="G12" s="472" t="n"/>
-      <c r="H12" s="472" t="n"/>
-      <c r="I12" s="473" t="n"/>
+      <c r="C12" s="432" t="n"/>
+      <c r="D12" s="432" t="n"/>
+      <c r="E12" s="432" t="n"/>
+      <c r="F12" s="432" t="n"/>
+      <c r="G12" s="432" t="n"/>
+      <c r="H12" s="432" t="n"/>
+      <c r="I12" s="433" t="n"/>
       <c r="J12" s="232" t="inlineStr">
         <is>
           <t>Mass/Lunch</t>
         </is>
       </c>
-      <c r="K12" s="474" t="n"/>
-      <c r="L12" s="474" t="n"/>
-      <c r="M12" s="474" t="n"/>
-      <c r="N12" s="474" t="n"/>
-      <c r="O12" s="474" t="n"/>
-      <c r="P12" s="474" t="n"/>
-      <c r="Q12" s="475" t="n"/>
+      <c r="K12" s="434" t="n"/>
+      <c r="L12" s="434" t="n"/>
+      <c r="M12" s="434" t="n"/>
+      <c r="N12" s="434" t="n"/>
+      <c r="O12" s="434" t="n"/>
+      <c r="P12" s="434" t="n"/>
+      <c r="Q12" s="435" t="n"/>
       <c r="R12" s="232" t="inlineStr">
         <is>
           <t>Mass/Lunch</t>
         </is>
       </c>
-      <c r="S12" s="474" t="n"/>
-      <c r="T12" s="474" t="n"/>
-      <c r="U12" s="474" t="n"/>
-      <c r="V12" s="474" t="n"/>
-      <c r="W12" s="474" t="n"/>
-      <c r="X12" s="474" t="n"/>
-      <c r="Y12" s="475" t="n"/>
+      <c r="S12" s="434" t="n"/>
+      <c r="T12" s="434" t="n"/>
+      <c r="U12" s="434" t="n"/>
+      <c r="V12" s="434" t="n"/>
+      <c r="W12" s="434" t="n"/>
+      <c r="X12" s="434" t="n"/>
+      <c r="Y12" s="435" t="n"/>
       <c r="Z12" s="232" t="inlineStr">
         <is>
           <t>Mass/Lunch</t>
         </is>
       </c>
-      <c r="AA12" s="474" t="n"/>
-      <c r="AB12" s="474" t="n"/>
-      <c r="AC12" s="474" t="n"/>
-      <c r="AD12" s="474" t="n"/>
-      <c r="AE12" s="474" t="n"/>
-      <c r="AF12" s="474" t="n"/>
-      <c r="AG12" s="475" t="n"/>
+      <c r="AA12" s="434" t="n"/>
+      <c r="AB12" s="434" t="n"/>
+      <c r="AC12" s="434" t="n"/>
+      <c r="AD12" s="434" t="n"/>
+      <c r="AE12" s="434" t="n"/>
+      <c r="AF12" s="434" t="n"/>
+      <c r="AG12" s="435" t="n"/>
       <c r="AH12" s="232" t="inlineStr">
         <is>
           <t>Mass/Lunch</t>
         </is>
       </c>
-      <c r="AI12" s="474" t="n"/>
-      <c r="AJ12" s="474" t="n"/>
-      <c r="AK12" s="474" t="n"/>
-      <c r="AL12" s="474" t="n"/>
-      <c r="AM12" s="474" t="n"/>
-      <c r="AN12" s="474" t="n"/>
-      <c r="AO12" s="475" t="n"/>
-      <c r="AP12" s="471" t="inlineStr">
+      <c r="AI12" s="434" t="n"/>
+      <c r="AJ12" s="434" t="n"/>
+      <c r="AK12" s="434" t="n"/>
+      <c r="AL12" s="434" t="n"/>
+      <c r="AM12" s="434" t="n"/>
+      <c r="AN12" s="434" t="n"/>
+      <c r="AO12" s="435" t="n"/>
+      <c r="AP12" s="431" t="inlineStr">
         <is>
           <t>12.00 PM - 1.30PM</t>
         </is>
@@ -4557,46 +4415,46 @@
           <t>1.30 PM - 2.20PM</t>
         </is>
       </c>
-      <c r="B14" s="152" t="n"/>
-      <c r="C14" s="424" t="n"/>
-      <c r="D14" s="435" t="n"/>
-      <c r="E14" s="425" t="n"/>
-      <c r="F14" s="425" t="n"/>
-      <c r="G14" s="476" t="n"/>
-      <c r="H14" s="424" t="n"/>
-      <c r="I14" s="426" t="n"/>
-      <c r="J14" s="427" t="n"/>
-      <c r="K14" s="428" t="n"/>
-      <c r="L14" s="430" t="n"/>
-      <c r="M14" s="428" t="n"/>
-      <c r="N14" s="429" t="n"/>
-      <c r="O14" s="430" t="n"/>
-      <c r="P14" s="430" t="n"/>
-      <c r="Q14" s="431" t="n"/>
-      <c r="R14" s="432" t="n"/>
-      <c r="S14" s="425" t="n"/>
-      <c r="T14" s="477" t="n"/>
-      <c r="U14" s="436" t="n"/>
-      <c r="V14" s="433" t="n"/>
-      <c r="W14" s="478" t="n"/>
-      <c r="X14" s="425" t="n"/>
-      <c r="Y14" s="479" t="n"/>
-      <c r="Z14" s="427" t="n"/>
-      <c r="AA14" s="428" t="n"/>
-      <c r="AB14" s="428" t="n"/>
-      <c r="AC14" s="429" t="n"/>
-      <c r="AD14" s="430" t="n"/>
-      <c r="AE14" s="428" t="n"/>
-      <c r="AF14" s="430" t="n"/>
-      <c r="AG14" s="431" t="n"/>
-      <c r="AH14" s="435" t="n"/>
-      <c r="AI14" s="425" t="n"/>
-      <c r="AJ14" s="436" t="n"/>
-      <c r="AK14" s="152" t="n"/>
-      <c r="AL14" s="151" t="n"/>
-      <c r="AM14" s="424" t="n"/>
-      <c r="AN14" s="425" t="n"/>
-      <c r="AO14" s="426" t="n"/>
+      <c r="B14" s="423" t="n"/>
+      <c r="C14" s="423" t="n"/>
+      <c r="D14" s="423" t="n"/>
+      <c r="E14" s="423" t="n"/>
+      <c r="F14" s="423" t="n"/>
+      <c r="G14" s="423" t="n"/>
+      <c r="H14" s="423" t="n"/>
+      <c r="I14" s="423" t="n"/>
+      <c r="J14" s="424" t="n"/>
+      <c r="K14" s="424" t="n"/>
+      <c r="L14" s="424" t="n"/>
+      <c r="M14" s="424" t="n"/>
+      <c r="N14" s="424" t="n"/>
+      <c r="O14" s="424" t="n"/>
+      <c r="P14" s="424" t="n"/>
+      <c r="Q14" s="424" t="n"/>
+      <c r="R14" s="423" t="n"/>
+      <c r="S14" s="423" t="n"/>
+      <c r="T14" s="423" t="n"/>
+      <c r="U14" s="423" t="n"/>
+      <c r="V14" s="423" t="n"/>
+      <c r="W14" s="423" t="n"/>
+      <c r="X14" s="423" t="n"/>
+      <c r="Y14" s="423" t="n"/>
+      <c r="Z14" s="424" t="n"/>
+      <c r="AA14" s="424" t="n"/>
+      <c r="AB14" s="424" t="n"/>
+      <c r="AC14" s="424" t="n"/>
+      <c r="AD14" s="424" t="n"/>
+      <c r="AE14" s="424" t="n"/>
+      <c r="AF14" s="424" t="n"/>
+      <c r="AG14" s="424" t="n"/>
+      <c r="AH14" s="423" t="n"/>
+      <c r="AI14" s="423" t="n"/>
+      <c r="AJ14" s="423" t="n"/>
+      <c r="AK14" s="423" t="n"/>
+      <c r="AL14" s="423" t="n"/>
+      <c r="AM14" s="423" t="n"/>
+      <c r="AN14" s="423" t="n"/>
+      <c r="AO14" s="423" t="n"/>
       <c r="AP14" s="422" t="inlineStr">
         <is>
           <t>1.30 PM - 2.20PM</t>
@@ -4604,336 +4462,336 @@
       </c>
     </row>
     <row r="15" ht="45.95" customHeight="1" thickBot="1">
-      <c r="A15" s="437" t="n"/>
-      <c r="B15" s="443" t="n"/>
-      <c r="C15" s="439" t="n"/>
-      <c r="D15" s="442" t="n"/>
-      <c r="E15" s="440" t="n"/>
-      <c r="F15" s="440" t="n"/>
-      <c r="G15" s="439" t="n"/>
-      <c r="H15" s="439" t="n"/>
-      <c r="I15" s="441" t="n"/>
-      <c r="J15" s="442" t="n"/>
-      <c r="K15" s="440" t="n"/>
-      <c r="L15" s="439" t="n"/>
-      <c r="M15" s="440" t="n"/>
-      <c r="N15" s="444" t="n"/>
-      <c r="O15" s="439" t="n"/>
-      <c r="P15" s="439" t="n"/>
-      <c r="Q15" s="441" t="n"/>
-      <c r="R15" s="441" t="n"/>
-      <c r="S15" s="440" t="n"/>
-      <c r="T15" s="439" t="n"/>
-      <c r="U15" s="444" t="n"/>
-      <c r="V15" s="440" t="n"/>
-      <c r="W15" s="438" t="n"/>
-      <c r="X15" s="440" t="n"/>
-      <c r="Y15" s="480" t="n"/>
-      <c r="Z15" s="442" t="n"/>
-      <c r="AA15" s="440" t="n"/>
-      <c r="AB15" s="440" t="n"/>
-      <c r="AC15" s="444" t="n"/>
-      <c r="AD15" s="439" t="n"/>
-      <c r="AE15" s="440" t="n"/>
-      <c r="AF15" s="439" t="n"/>
-      <c r="AG15" s="441" t="n"/>
-      <c r="AH15" s="442" t="n"/>
-      <c r="AI15" s="440" t="n"/>
-      <c r="AJ15" s="444" t="n"/>
-      <c r="AK15" s="443" t="n"/>
+      <c r="A15" s="425" t="n"/>
+      <c r="B15" s="421" t="n"/>
+      <c r="C15" s="421" t="n"/>
+      <c r="D15" s="421" t="n"/>
+      <c r="E15" s="421" t="n"/>
+      <c r="F15" s="421" t="n"/>
+      <c r="G15" s="421" t="n"/>
+      <c r="H15" s="421" t="n"/>
+      <c r="I15" s="421" t="n"/>
+      <c r="J15" s="421" t="n"/>
+      <c r="K15" s="421" t="n"/>
+      <c r="L15" s="421" t="n"/>
+      <c r="M15" s="421" t="n"/>
+      <c r="N15" s="421" t="n"/>
+      <c r="O15" s="421" t="n"/>
+      <c r="P15" s="421" t="n"/>
+      <c r="Q15" s="421" t="n"/>
+      <c r="R15" s="421" t="n"/>
+      <c r="S15" s="421" t="n"/>
+      <c r="T15" s="421" t="n"/>
+      <c r="U15" s="421" t="n"/>
+      <c r="V15" s="421" t="n"/>
+      <c r="W15" s="421" t="n"/>
+      <c r="X15" s="421" t="n"/>
+      <c r="Y15" s="421" t="n"/>
+      <c r="Z15" s="421" t="n"/>
+      <c r="AA15" s="421" t="n"/>
+      <c r="AB15" s="421" t="n"/>
+      <c r="AC15" s="421" t="n"/>
+      <c r="AD15" s="421" t="n"/>
+      <c r="AE15" s="421" t="n"/>
+      <c r="AF15" s="421" t="n"/>
+      <c r="AG15" s="421" t="n"/>
+      <c r="AH15" s="421" t="n"/>
+      <c r="AI15" s="421" t="n"/>
+      <c r="AJ15" s="421" t="n"/>
+      <c r="AK15" s="421" t="n"/>
       <c r="AL15" s="421" t="n"/>
-      <c r="AM15" s="439" t="n"/>
-      <c r="AN15" s="440" t="n"/>
-      <c r="AO15" s="441" t="n"/>
-      <c r="AP15" s="437" t="n"/>
+      <c r="AM15" s="421" t="n"/>
+      <c r="AN15" s="421" t="n"/>
+      <c r="AO15" s="421" t="n"/>
+      <c r="AP15" s="425" t="n"/>
     </row>
     <row r="16" ht="45.95" customHeight="1" thickBot="1">
-      <c r="A16" s="445" t="inlineStr">
+      <c r="A16" s="426" t="inlineStr">
         <is>
           <t>2.30 PM - 3.20 PM</t>
         </is>
       </c>
       <c r="B16" s="423" t="n"/>
-      <c r="C16" s="424" t="n"/>
-      <c r="D16" s="425" t="n"/>
-      <c r="E16" s="436" t="n"/>
-      <c r="F16" s="425" t="n"/>
-      <c r="G16" s="425" t="n"/>
-      <c r="H16" s="424" t="n"/>
-      <c r="I16" s="426" t="n"/>
-      <c r="J16" s="467" t="n"/>
-      <c r="K16" s="450" t="n"/>
-      <c r="L16" s="430" t="n"/>
-      <c r="M16" s="481" t="n"/>
-      <c r="N16" s="428" t="n"/>
-      <c r="O16" s="464" t="n"/>
-      <c r="P16" s="428" t="n"/>
-      <c r="Q16" s="431" t="n"/>
-      <c r="R16" s="482" t="n"/>
-      <c r="S16" s="425" t="n"/>
-      <c r="T16" s="456" t="n"/>
-      <c r="U16" s="425" t="n"/>
-      <c r="V16" s="483" t="n"/>
-      <c r="W16" s="424" t="n"/>
-      <c r="X16" s="436" t="n"/>
-      <c r="Y16" s="426" t="n"/>
-      <c r="Z16" s="448" t="n"/>
-      <c r="AA16" s="428" t="n"/>
-      <c r="AB16" s="430" t="n"/>
-      <c r="AC16" s="429" t="n"/>
-      <c r="AD16" s="449" t="n"/>
-      <c r="AE16" s="428" t="n"/>
-      <c r="AF16" s="430" t="n"/>
-      <c r="AG16" s="431" t="n"/>
-      <c r="AH16" s="435" t="n"/>
-      <c r="AI16" s="425" t="n"/>
-      <c r="AJ16" s="436" t="n"/>
-      <c r="AK16" s="152" t="n"/>
-      <c r="AL16" s="151" t="n"/>
-      <c r="AM16" s="424" t="n"/>
-      <c r="AN16" s="425" t="n"/>
-      <c r="AO16" s="426" t="n"/>
-      <c r="AP16" s="445" t="inlineStr">
+      <c r="C16" s="423" t="n"/>
+      <c r="D16" s="423" t="n"/>
+      <c r="E16" s="423" t="n"/>
+      <c r="F16" s="423" t="n"/>
+      <c r="G16" s="423" t="n"/>
+      <c r="H16" s="423" t="n"/>
+      <c r="I16" s="423" t="n"/>
+      <c r="J16" s="428" t="n"/>
+      <c r="K16" s="428" t="n"/>
+      <c r="L16" s="424" t="n"/>
+      <c r="M16" s="424" t="n"/>
+      <c r="N16" s="424" t="n"/>
+      <c r="O16" s="428" t="n"/>
+      <c r="P16" s="424" t="n"/>
+      <c r="Q16" s="424" t="n"/>
+      <c r="R16" s="427" t="n"/>
+      <c r="S16" s="423" t="n"/>
+      <c r="T16" s="427" t="n"/>
+      <c r="U16" s="423" t="n"/>
+      <c r="V16" s="423" t="n"/>
+      <c r="W16" s="423" t="n"/>
+      <c r="X16" s="423" t="n"/>
+      <c r="Y16" s="423" t="n"/>
+      <c r="Z16" s="424" t="n"/>
+      <c r="AA16" s="424" t="n"/>
+      <c r="AB16" s="424" t="n"/>
+      <c r="AC16" s="424" t="n"/>
+      <c r="AD16" s="424" t="n"/>
+      <c r="AE16" s="424" t="n"/>
+      <c r="AF16" s="424" t="n"/>
+      <c r="AG16" s="424" t="n"/>
+      <c r="AH16" s="423" t="n"/>
+      <c r="AI16" s="423" t="n"/>
+      <c r="AJ16" s="423" t="n"/>
+      <c r="AK16" s="423" t="n"/>
+      <c r="AL16" s="423" t="n"/>
+      <c r="AM16" s="423" t="n"/>
+      <c r="AN16" s="423" t="n"/>
+      <c r="AO16" s="423" t="n"/>
+      <c r="AP16" s="426" t="inlineStr">
         <is>
           <t>2.30 PM - 3.20 PM</t>
         </is>
       </c>
     </row>
     <row r="17" ht="45.95" customHeight="1" thickBot="1">
-      <c r="A17" s="437" t="n"/>
-      <c r="B17" s="438" t="n"/>
-      <c r="C17" s="439" t="n"/>
-      <c r="D17" s="440" t="n"/>
-      <c r="E17" s="444" t="n"/>
-      <c r="F17" s="440" t="n"/>
-      <c r="G17" s="440" t="n"/>
-      <c r="H17" s="439" t="n"/>
-      <c r="I17" s="441" t="n"/>
-      <c r="J17" s="470" t="n"/>
-      <c r="K17" s="457" t="n"/>
-      <c r="L17" s="439" t="n"/>
-      <c r="M17" s="440" t="n"/>
-      <c r="N17" s="440" t="n"/>
-      <c r="O17" s="456" t="n"/>
-      <c r="P17" s="440" t="n"/>
-      <c r="Q17" s="441" t="n"/>
-      <c r="R17" s="468" t="n"/>
-      <c r="S17" s="440" t="n"/>
-      <c r="T17" s="456" t="n"/>
-      <c r="U17" s="440" t="n"/>
-      <c r="V17" s="440" t="n"/>
-      <c r="W17" s="439" t="n"/>
-      <c r="X17" s="444" t="n"/>
-      <c r="Y17" s="441" t="n"/>
-      <c r="Z17" s="438" t="n"/>
-      <c r="AA17" s="440" t="n"/>
-      <c r="AB17" s="439" t="n"/>
-      <c r="AC17" s="444" t="n"/>
+      <c r="A17" s="425" t="n"/>
+      <c r="B17" s="421" t="n"/>
+      <c r="C17" s="421" t="n"/>
+      <c r="D17" s="421" t="n"/>
+      <c r="E17" s="421" t="n"/>
+      <c r="F17" s="421" t="n"/>
+      <c r="G17" s="421" t="n"/>
+      <c r="H17" s="421" t="n"/>
+      <c r="I17" s="421" t="n"/>
+      <c r="J17" s="429" t="n"/>
+      <c r="K17" s="429" t="n"/>
+      <c r="L17" s="421" t="n"/>
+      <c r="M17" s="421" t="n"/>
+      <c r="N17" s="421" t="n"/>
+      <c r="O17" s="429" t="n"/>
+      <c r="P17" s="421" t="n"/>
+      <c r="Q17" s="421" t="n"/>
+      <c r="R17" s="429" t="n"/>
+      <c r="S17" s="421" t="n"/>
+      <c r="T17" s="429" t="n"/>
+      <c r="U17" s="421" t="n"/>
+      <c r="V17" s="421" t="n"/>
+      <c r="W17" s="421" t="n"/>
+      <c r="X17" s="421" t="n"/>
+      <c r="Y17" s="421" t="n"/>
+      <c r="Z17" s="421" t="n"/>
+      <c r="AA17" s="421" t="n"/>
+      <c r="AB17" s="421" t="n"/>
+      <c r="AC17" s="421" t="n"/>
       <c r="AD17" s="421" t="n"/>
-      <c r="AE17" s="440" t="n"/>
-      <c r="AF17" s="439" t="n"/>
-      <c r="AG17" s="441" t="n"/>
-      <c r="AH17" s="442" t="n"/>
-      <c r="AI17" s="440" t="n"/>
-      <c r="AJ17" s="444" t="n"/>
-      <c r="AK17" s="443" t="n"/>
+      <c r="AE17" s="421" t="n"/>
+      <c r="AF17" s="421" t="n"/>
+      <c r="AG17" s="421" t="n"/>
+      <c r="AH17" s="421" t="n"/>
+      <c r="AI17" s="421" t="n"/>
+      <c r="AJ17" s="421" t="n"/>
+      <c r="AK17" s="421" t="n"/>
       <c r="AL17" s="421" t="n"/>
-      <c r="AM17" s="439" t="n"/>
-      <c r="AN17" s="440" t="n"/>
-      <c r="AO17" s="441" t="n"/>
-      <c r="AP17" s="437" t="n"/>
+      <c r="AM17" s="421" t="n"/>
+      <c r="AN17" s="421" t="n"/>
+      <c r="AO17" s="421" t="n"/>
+      <c r="AP17" s="425" t="n"/>
     </row>
     <row r="18" ht="45.95" customHeight="1">
-      <c r="A18" s="445" t="inlineStr">
+      <c r="A18" s="426" t="inlineStr">
         <is>
           <t>3.30 PM - 4.20 PM</t>
         </is>
       </c>
-      <c r="B18" s="446" t="n"/>
-      <c r="C18" s="424" t="n"/>
-      <c r="D18" s="424" t="n"/>
-      <c r="E18" s="478" t="n"/>
-      <c r="F18" s="426" t="n"/>
-      <c r="G18" s="451" t="n"/>
-      <c r="H18" s="424" t="n"/>
-      <c r="I18" s="426" t="n"/>
-      <c r="J18" s="427" t="n"/>
-      <c r="K18" s="428" t="n"/>
-      <c r="L18" s="429" t="n"/>
-      <c r="M18" s="428" t="n"/>
-      <c r="N18" s="452" t="n"/>
-      <c r="O18" s="481" t="n"/>
-      <c r="P18" s="428" t="n"/>
-      <c r="Q18" s="465" t="n"/>
-      <c r="R18" s="482" t="n"/>
-      <c r="S18" s="451" t="n"/>
-      <c r="T18" s="424" t="n"/>
-      <c r="U18" s="425" t="n"/>
-      <c r="V18" s="147" t="n"/>
-      <c r="W18" s="425" t="n"/>
-      <c r="X18" s="425" t="n"/>
-      <c r="Y18" s="426" t="n"/>
-      <c r="Z18" s="448" t="n"/>
-      <c r="AA18" s="450" t="n"/>
-      <c r="AB18" s="484" t="n"/>
-      <c r="AC18" s="485" t="n"/>
-      <c r="AD18" s="430" t="n"/>
-      <c r="AE18" s="428" t="n"/>
-      <c r="AF18" s="430" t="n"/>
-      <c r="AG18" s="431" t="n"/>
-      <c r="AH18" s="435" t="n"/>
-      <c r="AI18" s="425" t="n"/>
-      <c r="AJ18" s="436" t="n"/>
-      <c r="AK18" s="453" t="n"/>
-      <c r="AL18" s="424" t="n"/>
-      <c r="AM18" s="425" t="n"/>
-      <c r="AN18" s="425" t="n"/>
-      <c r="AO18" s="426" t="n"/>
-      <c r="AP18" s="445" t="inlineStr">
+      <c r="B18" s="427" t="n"/>
+      <c r="C18" s="423" t="n"/>
+      <c r="D18" s="423" t="n"/>
+      <c r="E18" s="423" t="n"/>
+      <c r="F18" s="423" t="n"/>
+      <c r="G18" s="427" t="n"/>
+      <c r="H18" s="423" t="n"/>
+      <c r="I18" s="423" t="n"/>
+      <c r="J18" s="424" t="n"/>
+      <c r="K18" s="424" t="n"/>
+      <c r="L18" s="424" t="n"/>
+      <c r="M18" s="424" t="n"/>
+      <c r="N18" s="428" t="n"/>
+      <c r="O18" s="424" t="n"/>
+      <c r="P18" s="424" t="n"/>
+      <c r="Q18" s="428" t="n"/>
+      <c r="R18" s="427" t="n"/>
+      <c r="S18" s="427" t="n"/>
+      <c r="T18" s="423" t="n"/>
+      <c r="U18" s="423" t="n"/>
+      <c r="V18" s="423" t="n"/>
+      <c r="W18" s="423" t="n"/>
+      <c r="X18" s="423" t="n"/>
+      <c r="Y18" s="423" t="n"/>
+      <c r="Z18" s="424" t="n"/>
+      <c r="AA18" s="428" t="n"/>
+      <c r="AB18" s="424" t="n"/>
+      <c r="AC18" s="424" t="n"/>
+      <c r="AD18" s="424" t="n"/>
+      <c r="AE18" s="424" t="n"/>
+      <c r="AF18" s="424" t="n"/>
+      <c r="AG18" s="424" t="n"/>
+      <c r="AH18" s="423" t="n"/>
+      <c r="AI18" s="423" t="n"/>
+      <c r="AJ18" s="423" t="n"/>
+      <c r="AK18" s="427" t="n"/>
+      <c r="AL18" s="423" t="n"/>
+      <c r="AM18" s="423" t="n"/>
+      <c r="AN18" s="423" t="n"/>
+      <c r="AO18" s="423" t="n"/>
+      <c r="AP18" s="426" t="inlineStr">
         <is>
           <t>3.30 PM - 4.20 PM</t>
         </is>
       </c>
     </row>
     <row r="19" ht="45.95" customHeight="1" thickBot="1">
-      <c r="A19" s="437" t="n"/>
-      <c r="B19" s="455" t="n"/>
-      <c r="C19" s="439" t="n"/>
-      <c r="D19" s="439" t="n"/>
-      <c r="E19" s="438" t="n"/>
-      <c r="F19" s="441" t="n"/>
-      <c r="G19" s="457" t="n"/>
-      <c r="H19" s="439" t="n"/>
-      <c r="I19" s="441" t="n"/>
-      <c r="J19" s="442" t="n"/>
-      <c r="K19" s="440" t="n"/>
-      <c r="L19" s="444" t="n"/>
-      <c r="M19" s="440" t="n"/>
-      <c r="N19" s="459" t="n"/>
-      <c r="O19" s="440" t="n"/>
-      <c r="P19" s="440" t="n"/>
-      <c r="Q19" s="468" t="n"/>
-      <c r="R19" s="468" t="n"/>
-      <c r="S19" s="457" t="n"/>
-      <c r="T19" s="439" t="n"/>
-      <c r="U19" s="440" t="n"/>
-      <c r="V19" s="440" t="n"/>
-      <c r="W19" s="440" t="n"/>
-      <c r="X19" s="440" t="n"/>
-      <c r="Y19" s="441" t="n"/>
-      <c r="Z19" s="438" t="n"/>
-      <c r="AA19" s="457" t="n"/>
-      <c r="AB19" s="469" t="n"/>
+      <c r="A19" s="425" t="n"/>
+      <c r="B19" s="429" t="n"/>
+      <c r="C19" s="421" t="n"/>
+      <c r="D19" s="421" t="n"/>
+      <c r="E19" s="421" t="n"/>
+      <c r="F19" s="421" t="n"/>
+      <c r="G19" s="429" t="n"/>
+      <c r="H19" s="421" t="n"/>
+      <c r="I19" s="421" t="n"/>
+      <c r="J19" s="421" t="n"/>
+      <c r="K19" s="421" t="n"/>
+      <c r="L19" s="421" t="n"/>
+      <c r="M19" s="421" t="n"/>
+      <c r="N19" s="429" t="n"/>
+      <c r="O19" s="421" t="n"/>
+      <c r="P19" s="421" t="n"/>
+      <c r="Q19" s="429" t="n"/>
+      <c r="R19" s="429" t="n"/>
+      <c r="S19" s="429" t="n"/>
+      <c r="T19" s="421" t="n"/>
+      <c r="U19" s="421" t="n"/>
+      <c r="V19" s="421" t="n"/>
+      <c r="W19" s="421" t="n"/>
+      <c r="X19" s="421" t="n"/>
+      <c r="Y19" s="421" t="n"/>
+      <c r="Z19" s="421" t="n"/>
+      <c r="AA19" s="429" t="n"/>
+      <c r="AB19" s="421" t="n"/>
       <c r="AC19" s="421" t="n"/>
-      <c r="AD19" s="439" t="n"/>
-      <c r="AE19" s="440" t="n"/>
-      <c r="AF19" s="439" t="n"/>
-      <c r="AG19" s="441" t="n"/>
-      <c r="AH19" s="442" t="n"/>
-      <c r="AI19" s="440" t="n"/>
-      <c r="AJ19" s="444" t="n"/>
-      <c r="AK19" s="460" t="n"/>
-      <c r="AL19" s="439" t="n"/>
-      <c r="AM19" s="440" t="n"/>
-      <c r="AN19" s="440" t="n"/>
-      <c r="AO19" s="441" t="n"/>
-      <c r="AP19" s="437" t="n"/>
+      <c r="AD19" s="421" t="n"/>
+      <c r="AE19" s="421" t="n"/>
+      <c r="AF19" s="421" t="n"/>
+      <c r="AG19" s="421" t="n"/>
+      <c r="AH19" s="421" t="n"/>
+      <c r="AI19" s="421" t="n"/>
+      <c r="AJ19" s="421" t="n"/>
+      <c r="AK19" s="429" t="n"/>
+      <c r="AL19" s="421" t="n"/>
+      <c r="AM19" s="421" t="n"/>
+      <c r="AN19" s="421" t="n"/>
+      <c r="AO19" s="421" t="n"/>
+      <c r="AP19" s="425" t="n"/>
     </row>
     <row r="20" ht="45.95" customHeight="1">
-      <c r="A20" s="445" t="inlineStr">
+      <c r="A20" s="426" t="inlineStr">
         <is>
           <t>4.30 PM - 5.20 PM</t>
         </is>
       </c>
-      <c r="B20" s="435" t="n"/>
-      <c r="C20" s="425" t="n"/>
-      <c r="D20" s="424" t="n"/>
-      <c r="E20" s="478" t="n"/>
-      <c r="F20" s="426" t="n"/>
-      <c r="G20" s="451" t="n"/>
-      <c r="H20" s="425" t="n"/>
-      <c r="I20" s="486" t="n"/>
-      <c r="J20" s="427" t="n"/>
-      <c r="K20" s="428" t="n"/>
-      <c r="L20" s="429" t="n"/>
-      <c r="M20" s="428" t="n"/>
-      <c r="N20" s="430" t="n"/>
-      <c r="O20" s="428" t="n"/>
-      <c r="P20" s="428" t="n"/>
-      <c r="Q20" s="431" t="n"/>
-      <c r="R20" s="435" t="n"/>
-      <c r="S20" s="425" t="n"/>
-      <c r="T20" s="425" t="n"/>
-      <c r="U20" s="433" t="n"/>
-      <c r="V20" s="424" t="n"/>
-      <c r="W20" s="425" t="n"/>
-      <c r="X20" s="425" t="n"/>
-      <c r="Y20" s="487" t="n"/>
-      <c r="Z20" s="448" t="n"/>
-      <c r="AA20" s="450" t="n"/>
-      <c r="AB20" s="484" t="n"/>
-      <c r="AC20" s="158" t="n"/>
-      <c r="AD20" s="464" t="n"/>
-      <c r="AE20" s="428" t="n"/>
-      <c r="AF20" s="428" t="n"/>
-      <c r="AG20" s="431" t="n"/>
-      <c r="AH20" s="435" t="n"/>
-      <c r="AI20" s="425" t="n"/>
-      <c r="AJ20" s="436" t="n"/>
-      <c r="AK20" s="453" t="n"/>
-      <c r="AL20" s="424" t="n"/>
-      <c r="AM20" s="425" t="n"/>
-      <c r="AN20" s="425" t="n"/>
-      <c r="AO20" s="426" t="n"/>
-      <c r="AP20" s="445" t="inlineStr">
+      <c r="B20" s="423" t="n"/>
+      <c r="C20" s="423" t="n"/>
+      <c r="D20" s="423" t="n"/>
+      <c r="E20" s="423" t="n"/>
+      <c r="F20" s="423" t="n"/>
+      <c r="G20" s="427" t="n"/>
+      <c r="H20" s="423" t="n"/>
+      <c r="I20" s="427" t="n"/>
+      <c r="J20" s="424" t="n"/>
+      <c r="K20" s="424" t="n"/>
+      <c r="L20" s="424" t="n"/>
+      <c r="M20" s="424" t="n"/>
+      <c r="N20" s="424" t="n"/>
+      <c r="O20" s="424" t="n"/>
+      <c r="P20" s="424" t="n"/>
+      <c r="Q20" s="424" t="n"/>
+      <c r="R20" s="423" t="n"/>
+      <c r="S20" s="423" t="n"/>
+      <c r="T20" s="423" t="n"/>
+      <c r="U20" s="423" t="n"/>
+      <c r="V20" s="423" t="n"/>
+      <c r="W20" s="423" t="n"/>
+      <c r="X20" s="423" t="n"/>
+      <c r="Y20" s="427" t="n"/>
+      <c r="Z20" s="424" t="n"/>
+      <c r="AA20" s="428" t="n"/>
+      <c r="AB20" s="424" t="n"/>
+      <c r="AC20" s="424" t="n"/>
+      <c r="AD20" s="428" t="n"/>
+      <c r="AE20" s="424" t="n"/>
+      <c r="AF20" s="424" t="n"/>
+      <c r="AG20" s="424" t="n"/>
+      <c r="AH20" s="423" t="n"/>
+      <c r="AI20" s="423" t="n"/>
+      <c r="AJ20" s="423" t="n"/>
+      <c r="AK20" s="427" t="n"/>
+      <c r="AL20" s="423" t="n"/>
+      <c r="AM20" s="423" t="n"/>
+      <c r="AN20" s="423" t="n"/>
+      <c r="AO20" s="423" t="n"/>
+      <c r="AP20" s="426" t="inlineStr">
         <is>
           <t>4.30 PM - 5.20 PM</t>
         </is>
       </c>
     </row>
     <row r="21" ht="45.95" customHeight="1" thickBot="1">
-      <c r="A21" s="437" t="n"/>
-      <c r="B21" s="442" t="n"/>
-      <c r="C21" s="440" t="n"/>
-      <c r="D21" s="439" t="n"/>
-      <c r="E21" s="438" t="n"/>
-      <c r="F21" s="441" t="n"/>
-      <c r="G21" s="457" t="n"/>
-      <c r="H21" s="440" t="n"/>
-      <c r="I21" s="468" t="n"/>
-      <c r="J21" s="442" t="n"/>
-      <c r="K21" s="440" t="n"/>
-      <c r="L21" s="444" t="n"/>
-      <c r="M21" s="440" t="n"/>
-      <c r="N21" s="439" t="n"/>
-      <c r="O21" s="440" t="n"/>
-      <c r="P21" s="440" t="n"/>
-      <c r="Q21" s="441" t="n"/>
-      <c r="R21" s="442" t="n"/>
-      <c r="S21" s="440" t="n"/>
-      <c r="T21" s="440" t="n"/>
-      <c r="U21" s="440" t="n"/>
-      <c r="V21" s="439" t="n"/>
-      <c r="W21" s="440" t="n"/>
-      <c r="X21" s="440" t="n"/>
-      <c r="Y21" s="468" t="n"/>
-      <c r="Z21" s="438" t="n"/>
-      <c r="AA21" s="457" t="n"/>
-      <c r="AB21" s="469" t="n"/>
+      <c r="A21" s="425" t="n"/>
+      <c r="B21" s="421" t="n"/>
+      <c r="C21" s="421" t="n"/>
+      <c r="D21" s="421" t="n"/>
+      <c r="E21" s="421" t="n"/>
+      <c r="F21" s="421" t="n"/>
+      <c r="G21" s="429" t="n"/>
+      <c r="H21" s="421" t="n"/>
+      <c r="I21" s="429" t="n"/>
+      <c r="J21" s="421" t="n"/>
+      <c r="K21" s="421" t="n"/>
+      <c r="L21" s="421" t="n"/>
+      <c r="M21" s="421" t="n"/>
+      <c r="N21" s="421" t="n"/>
+      <c r="O21" s="421" t="n"/>
+      <c r="P21" s="421" t="n"/>
+      <c r="Q21" s="421" t="n"/>
+      <c r="R21" s="421" t="n"/>
+      <c r="S21" s="421" t="n"/>
+      <c r="T21" s="421" t="n"/>
+      <c r="U21" s="421" t="n"/>
+      <c r="V21" s="421" t="n"/>
+      <c r="W21" s="421" t="n"/>
+      <c r="X21" s="421" t="n"/>
+      <c r="Y21" s="429" t="n"/>
+      <c r="Z21" s="421" t="n"/>
+      <c r="AA21" s="429" t="n"/>
+      <c r="AB21" s="421" t="n"/>
       <c r="AC21" s="421" t="n"/>
-      <c r="AD21" s="456" t="n"/>
-      <c r="AE21" s="440" t="n"/>
-      <c r="AF21" s="440" t="n"/>
-      <c r="AG21" s="441" t="n"/>
-      <c r="AH21" s="442" t="n"/>
-      <c r="AI21" s="440" t="n"/>
-      <c r="AJ21" s="444" t="n"/>
-      <c r="AK21" s="460" t="n"/>
-      <c r="AL21" s="439" t="n"/>
-      <c r="AM21" s="440" t="n"/>
-      <c r="AN21" s="440" t="n"/>
-      <c r="AO21" s="441" t="n"/>
-      <c r="AP21" s="437" t="n"/>
+      <c r="AD21" s="429" t="n"/>
+      <c r="AE21" s="421" t="n"/>
+      <c r="AF21" s="421" t="n"/>
+      <c r="AG21" s="421" t="n"/>
+      <c r="AH21" s="421" t="n"/>
+      <c r="AI21" s="421" t="n"/>
+      <c r="AJ21" s="421" t="n"/>
+      <c r="AK21" s="429" t="n"/>
+      <c r="AL21" s="421" t="n"/>
+      <c r="AM21" s="421" t="n"/>
+      <c r="AN21" s="421" t="n"/>
+      <c r="AO21" s="421" t="n"/>
+      <c r="AP21" s="425" t="n"/>
     </row>
     <row r="22" ht="45.95" customHeight="1">
       <c r="A22" s="99" t="n"/>
@@ -4961,7 +4819,7 @@
       <c r="W22" s="101" t="n"/>
       <c r="X22" s="101" t="n"/>
       <c r="Y22" s="103" t="n"/>
-      <c r="Z22" s="488" t="inlineStr">
+      <c r="Z22" s="436" t="inlineStr">
         <is>
           <t>FORMAL HALL</t>
         </is>
@@ -4972,7 +4830,7 @@
       <c r="AD22" s="414" t="n"/>
       <c r="AE22" s="414" t="n"/>
       <c r="AF22" s="414" t="n"/>
-      <c r="AG22" s="489" t="n"/>
+      <c r="AG22" s="437" t="n"/>
       <c r="AH22" s="100" t="n"/>
       <c r="AI22" s="101" t="n"/>
       <c r="AJ22" s="101" t="n"/>
@@ -5013,14 +4871,14 @@
       <c r="W23" s="105" t="n"/>
       <c r="X23" s="105" t="n"/>
       <c r="Y23" s="107" t="n"/>
-      <c r="Z23" s="490" t="n"/>
+      <c r="Z23" s="438" t="n"/>
       <c r="AA23" s="414" t="n"/>
       <c r="AB23" s="414" t="n"/>
       <c r="AC23" s="414" t="n"/>
       <c r="AD23" s="414" t="n"/>
       <c r="AE23" s="414" t="n"/>
       <c r="AF23" s="414" t="n"/>
-      <c r="AG23" s="489" t="n"/>
+      <c r="AG23" s="437" t="n"/>
       <c r="AH23" s="104" t="n"/>
       <c r="AI23" s="105" t="n"/>
       <c r="AJ23" s="105" t="n"/>
@@ -5061,14 +4919,14 @@
       <c r="W24" s="109" t="n"/>
       <c r="X24" s="109" t="n"/>
       <c r="Y24" s="110" t="n"/>
-      <c r="Z24" s="490" t="n"/>
+      <c r="Z24" s="438" t="n"/>
       <c r="AA24" s="414" t="n"/>
       <c r="AB24" s="414" t="n"/>
       <c r="AC24" s="414" t="n"/>
       <c r="AD24" s="414" t="n"/>
       <c r="AE24" s="414" t="n"/>
       <c r="AF24" s="414" t="n"/>
-      <c r="AG24" s="489" t="n"/>
+      <c r="AG24" s="437" t="n"/>
       <c r="AH24" s="108" t="n"/>
       <c r="AI24" s="109" t="n"/>
       <c r="AJ24" s="109" t="n"/>
@@ -5109,14 +4967,14 @@
       <c r="W25" s="105" t="n"/>
       <c r="X25" s="105" t="n"/>
       <c r="Y25" s="106" t="n"/>
-      <c r="Z25" s="438" t="n"/>
-      <c r="AA25" s="469" t="n"/>
-      <c r="AB25" s="469" t="n"/>
-      <c r="AC25" s="469" t="n"/>
-      <c r="AD25" s="469" t="n"/>
-      <c r="AE25" s="469" t="n"/>
-      <c r="AF25" s="469" t="n"/>
-      <c r="AG25" s="480" t="n"/>
+      <c r="Z25" s="439" t="n"/>
+      <c r="AA25" s="440" t="n"/>
+      <c r="AB25" s="440" t="n"/>
+      <c r="AC25" s="440" t="n"/>
+      <c r="AD25" s="440" t="n"/>
+      <c r="AE25" s="440" t="n"/>
+      <c r="AF25" s="440" t="n"/>
+      <c r="AG25" s="441" t="n"/>
       <c r="AH25" s="104" t="n"/>
       <c r="AI25" s="105" t="n"/>
       <c r="AJ25" s="105" t="n"/>

</xml_diff>